<commit_message>
food-delivery: spell out concrete UI steps for FE/UI cases in TestCases.xlsx (screen, URL, navigation, on-screen check)
</commit_message>
<xml_diff>
--- a/testcases/TestCases.xlsx
+++ b/testcases/TestCases.xlsx
@@ -6199,7 +6199,9 @@
       </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
-          <t>Then the home page lists the active restaurants, once each</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: the home page lists the active restaurants, once each.</t>
         </is>
       </c>
       <c r="H108" s="3" t="inlineStr">
@@ -6249,7 +6251,9 @@
       </c>
       <c r="G109" s="3" t="inlineStr">
         <is>
-          <t>Then the home page does not list restaurant 4</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: the home page does not list restaurant 4.</t>
         </is>
       </c>
       <c r="H109" s="3" t="inlineStr">
@@ -6299,7 +6303,9 @@
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>Then each home row links to its restaurant page</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: each home row links to its restaurant page.</t>
         </is>
       </c>
       <c r="H110" s="3" t="inlineStr">
@@ -6349,7 +6355,9 @@
       </c>
       <c r="G111" s="3" t="inlineStr">
         <is>
-          <t>Then the home page shows at least one restaurant</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: the home page shows at least one restaurant.</t>
         </is>
       </c>
       <c r="H111" s="3" t="inlineStr">
@@ -6399,8 +6407,10 @@
       </c>
       <c r="G112" s="3" t="inlineStr">
         <is>
-          <t>When the menu for restaurant 1 is opened
-Then every menu price on screen equals the item row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Restaurant menu' screen in the browser (URL /restaurant/1) — on Home, click restaurant 1.
+4. On screen, verify: every menu price on screen equals the item row.</t>
         </is>
       </c>
       <c r="H112" s="3" t="inlineStr">
@@ -6450,8 +6460,10 @@
       </c>
       <c r="G113" s="3" t="inlineStr">
         <is>
-          <t>When the menu for restaurant 1 is opened
-Then menu item 3 is shown unavailable</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Restaurant menu' screen in the browser (URL /restaurant/1) — on Home, click restaurant 1.
+4. On screen, verify: menu item 3 is shown unavailable.</t>
         </is>
       </c>
       <c r="H113" s="3" t="inlineStr">
@@ -6501,8 +6513,10 @@
       </c>
       <c r="G114" s="3" t="inlineStr">
         <is>
-          <t>When the menu for restaurant 1 is opened
-Then menu item 1 is shown available</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Restaurant menu' screen in the browser (URL /restaurant/1) — on Home, click restaurant 1.
+4. On screen, verify: menu item 1 is shown available.</t>
         </is>
       </c>
       <c r="H114" s="3" t="inlineStr">
@@ -6552,8 +6566,10 @@
       </c>
       <c r="G115" s="3" t="inlineStr">
         <is>
-          <t>When the menu for restaurant 2 is opened
-Then every menu price on screen is a dollar amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Restaurant menu' screen in the browser (URL /restaurant/2) — on Home, click restaurant 2.
+4. On screen, verify: every menu price on screen is a dollar amount.</t>
         </is>
       </c>
       <c r="H115" s="3" t="inlineStr">
@@ -6603,8 +6619,10 @@
       </c>
       <c r="G116" s="3" t="inlineStr">
         <is>
-          <t>When the menu for restaurant 3 is opened
-Then every menu name on screen equals the item row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Restaurant menu' screen in the browser (URL /restaurant/3) — on Home, click restaurant 3.
+4. On screen, verify: every menu name on screen equals the item row.</t>
         </is>
       </c>
       <c r="H116" s="3" t="inlineStr">
@@ -6654,8 +6672,10 @@
       </c>
       <c r="G117" s="3" t="inlineStr">
         <is>
-          <t>When the menu for restaurant 999 is opened
-Then the page reports not found</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Restaurant menu' screen in the browser (URL /restaurant/999) — on Home, click restaurant 999.
+4. On screen, verify: the page reports not found.</t>
         </is>
       </c>
       <c r="H117" s="3" t="inlineStr">
@@ -6705,8 +6725,10 @@
       </c>
       <c r="G118" s="3" t="inlineStr">
         <is>
-          <t>When the menu for restaurant &lt;rid&gt; is opened
-Then every menu price on screen equals the item row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): the menu for restaurant &lt;rid&gt; is opened.
+4. On screen, verify: every menu price on screen equals the item row.</t>
         </is>
       </c>
       <c r="H118" s="3" t="inlineStr">
@@ -6756,8 +6778,10 @@
       </c>
       <c r="G119" s="3" t="inlineStr">
         <is>
-          <t>When the menu for restaurant &lt;rid&gt; is opened
-Then every menu price on screen equals the item row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): the menu for restaurant &lt;rid&gt; is opened.
+4. On screen, verify: every menu price on screen equals the item row.</t>
         </is>
       </c>
       <c r="H119" s="3" t="inlineStr">
@@ -6807,8 +6831,10 @@
       </c>
       <c r="G120" s="3" t="inlineStr">
         <is>
-          <t>When the menu for restaurant &lt;rid&gt; is opened
-Then every menu price on screen equals the item row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): the menu for restaurant &lt;rid&gt; is opened.
+4. On screen, verify: every menu price on screen equals the item row.</t>
         </is>
       </c>
       <c r="H120" s="3" t="inlineStr">
@@ -6858,9 +6884,11 @@
       </c>
       <c r="G121" s="3" t="inlineStr">
         <is>
-          <t>Given a placed order of 2 of item 1 at restaurant 1
-When the order page is opened
-Then the order page total equals the stored order total</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a placed order of 2 of item 1 at restaurant 1.
+4. Open the app 'Order tracker' screen in the browser (URL /order/&lt;the placed order&gt;) — click the placed order.
+5. On screen, verify: the order page total equals the stored order total.</t>
         </is>
       </c>
       <c r="H121" s="3" t="inlineStr">
@@ -6910,9 +6938,11 @@
       </c>
       <c r="G122" s="3" t="inlineStr">
         <is>
-          <t>Given a placed order of 1 of item 1 at restaurant 1
-When the order page is opened
-Then the order page shows the order id and status "placed"</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a placed order of 1 of item 1 at restaurant 1.
+4. Open the app 'Order tracker' screen in the browser (URL /order/&lt;the placed order&gt;) — click the placed order.
+5. On screen, verify: the order page shows the order id and status "placed".</t>
         </is>
       </c>
       <c r="H122" s="3" t="inlineStr">
@@ -6962,9 +6992,11 @@
       </c>
       <c r="G123" s="3" t="inlineStr">
         <is>
-          <t>Given a placed order of 1 of item 5 at restaurant 2
-When the order page is opened
-Then the order page total is shown as a dollar amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a placed order of 1 of item 5 at restaurant 2.
+4. Open the app 'Order tracker' screen in the browser (URL /order/&lt;the placed order&gt;) — click the placed order.
+5. On screen, verify: the order page total is shown as a dollar amount.</t>
         </is>
       </c>
       <c r="H123" s="3" t="inlineStr">
@@ -7014,8 +7046,10 @@
       </c>
       <c r="G124" s="3" t="inlineStr">
         <is>
-          <t>When the order page for 999999 is opened
-Then the page reports not found</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Order tracker' screen in the browser (URL /order/999999) — open order 999999.
+4. On screen, verify: the page reports not found.</t>
         </is>
       </c>
       <c r="H124" s="3" t="inlineStr">
@@ -7065,9 +7099,11 @@
       </c>
       <c r="G125" s="3" t="inlineStr">
         <is>
-          <t>Given a delivered order of 1 of item 8 at restaurant 3
-When the order page is opened
-Then the order page shows status "delivered"</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a delivered order of 1 of item 8 at restaurant 3.
+4. Open the app 'Order tracker' screen in the browser (URL /order/&lt;the placed order&gt;) — click the placed order.
+5. On screen, verify: the order page shows status "delivered".</t>
         </is>
       </c>
       <c r="H125" s="3" t="inlineStr">
@@ -7117,9 +7153,11 @@
       </c>
       <c r="G126" s="3" t="inlineStr">
         <is>
-          <t>Given a placed order of 1 of item 1 at restaurant 1
-When the merchant board for restaurant 1 is opened
-Then the placed order appears on the merchant board with status "placed"</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a placed order of 1 of item 1 at restaurant 1.
+4. Open the app 'Merchant board' screen in the browser (URL /merchant/1) — open the merchant board for restaurant 1.
+5. On screen, verify: the placed order appears on the merchant board with status "placed".</t>
         </is>
       </c>
       <c r="H126" s="3" t="inlineStr">
@@ -7169,9 +7207,11 @@
       </c>
       <c r="G127" s="3" t="inlineStr">
         <is>
-          <t>Given a placed order of 1 of item 2 at restaurant 1
-When the merchant board for restaurant 1 is opened
-Then every order total on the board is a dollar amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a placed order of 1 of item 2 at restaurant 1.
+4. Open the app 'Merchant board' screen in the browser (URL /merchant/1) — open the merchant board for restaurant 1.
+5. On screen, verify: every order total on the board is a dollar amount.</t>
         </is>
       </c>
       <c r="H127" s="3" t="inlineStr">
@@ -7221,9 +7261,11 @@
       </c>
       <c r="G128" s="3" t="inlineStr">
         <is>
-          <t>Given a ready order of 1 of item 1 at restaurant 1
-When the driver board is opened
-Then the ready order is offered on the driver board</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a ready order of 1 of item 1 at restaurant 1.
+4. Open the app 'Driver board' screen in the browser (URL /driver/1) — open the driver board.
+5. On screen, verify: the ready order is offered on the driver board.</t>
         </is>
       </c>
       <c r="H128" s="3" t="inlineStr">
@@ -7273,9 +7315,11 @@
       </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>Given a ready order of 1 of item 5 at restaurant 2
-When the driver board is opened
-Then the driver board offer count equals the API offer count</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a ready order of 1 of item 5 at restaurant 2.
+4. Open the app 'Driver board' screen in the browser (URL /driver/1) — open the driver board.
+5. On screen, verify: the driver board offer count equals the API offer count.</t>
         </is>
       </c>
       <c r="H129" s="3" t="inlineStr">
@@ -7325,9 +7369,11 @@
       </c>
       <c r="G130" s="3" t="inlineStr">
         <is>
-          <t>Given a ready order of 1 of item 8 at restaurant 3
-When the driver board is opened
-Then every offered fee on the board is a dollar amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a ready order of 1 of item 8 at restaurant 3.
+4. Open the app 'Driver board' screen in the browser (URL /driver/1) — open the driver board.
+5. On screen, verify: every offered fee on the board is a dollar amount.</t>
         </is>
       </c>
       <c r="H130" s="3" t="inlineStr">
@@ -7377,8 +7423,10 @@
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>When the admin page is opened
-Then the admin revenue is shown as a dollar amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Admin overview' screen in the browser (URL /admin) — on Home, click 'Admin'.
+4. On screen, verify: the admin revenue is shown as a dollar amount.</t>
         </is>
       </c>
       <c r="H131" s="3" t="inlineStr">
@@ -7428,9 +7476,11 @@
       </c>
       <c r="G132" s="3" t="inlineStr">
         <is>
-          <t>Given a delivered order of 1 of item 1 at restaurant 1
-When the admin page is opened
-Then the admin page shows at least one delivered order</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a delivered order of 1 of item 1 at restaurant 1.
+4. Open the app 'Admin overview' screen in the browser (URL /admin) — on Home, click 'Admin'.
+5. On screen, verify: the admin page shows at least one delivered order.</t>
         </is>
       </c>
       <c r="H132" s="3" t="inlineStr">
@@ -7480,8 +7530,10 @@
       </c>
       <c r="G133" s="3" t="inlineStr">
         <is>
-          <t>When the admin page is opened
-Then every admin status count is a non-negative integer</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – restaurants' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Admin overview' screen in the browser (URL /admin) — on Home, click 'Admin'.
+4. On screen, verify: every admin status count is a non-negative integer.</t>
         </is>
       </c>
       <c r="H133" s="3" t="inlineStr">

</xml_diff>